<commit_message>
suppression de l'extension inseecodeextension (usage de discrict à la place 2f9e393188b7d985310ad064c55ef068893ac399
</commit_message>
<xml_diff>
--- a/ig/nr-update-FrAddress/StructureDefinition-fr-core-address.xlsx
+++ b/ig/nr-update-FrAddress/StructureDefinition-fr-core-address.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="161">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-10-16T08:20:44+00:00</t>
+    <t>2023-10-16T09:01:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -216,22 +216,6 @@
   </si>
   <si>
     <t>N/A</t>
-  </si>
-  <si>
-    <t>Address.extension:inseeCode</t>
-  </si>
-  <si>
-    <t>inseeCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {http://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-address-insee-code}
-</t>
-  </si>
-  <si>
-    <t>FR Core Address Insee Code Extension</t>
-  </si>
-  <si>
-    <t>This extension adds the insee code (5 digits) to the address | Ajout du code insee (5 chiffres) à l'adresse postale</t>
   </si>
   <si>
     <t>Address.use</t>
@@ -832,19 +816,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN14"/>
+  <dimension ref="A1:AN13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="19.28515625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="19.28515625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.62109375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="12.64453125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="6" max="6" width="2.2109375" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="2.2109375" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="2.1640625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="77.2890625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="10.04296875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -867,6 +850,7 @@
     <col min="32" max="32" width="19.28515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="2.2109375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="2.2109375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" hidden="true" width="8.0" customWidth="false"/>
     <col min="17" max="17" width="20.703125" customWidth="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
     <col min="37" max="37" width="107.3984375" customWidth="true" bestFit="true"/>
@@ -1220,11 +1204,9 @@
         <v>65</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>53</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>66</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
         <v>35</v>
       </c>
@@ -1239,10 +1221,10 @@
         <v>35</v>
       </c>
       <c r="I4" t="s" s="2">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="J4" t="s" s="2">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="K4" t="s" s="2">
         <v>67</v>
@@ -1253,8 +1235,12 @@
       <c r="M4" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="N4" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="O4" t="s" s="2">
+        <v>71</v>
+      </c>
       <c r="P4" t="s" s="2">
         <v>35</v>
       </c>
@@ -1266,7 +1252,7 @@
         <v>35</v>
       </c>
       <c r="T4" t="s" s="2">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="U4" t="s" s="2">
         <v>35</v>
@@ -1278,13 +1264,13 @@
         <v>35</v>
       </c>
       <c r="X4" t="s" s="2">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="Y4" t="s" s="2">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="Z4" t="s" s="2">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="AA4" t="s" s="2">
         <v>35</v>
@@ -1302,28 +1288,28 @@
         <v>35</v>
       </c>
       <c r="AF4" t="s" s="2">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH4" t="s" s="2">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="AI4" t="s" s="2">
         <v>42</v>
       </c>
       <c r="AJ4" t="s" s="2">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="AK4" t="s" s="2">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="AL4" t="s" s="2">
-        <v>35</v>
+        <v>77</v>
       </c>
       <c r="AM4" t="s" s="2">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="AN4" t="s" s="2">
         <v>35</v>
@@ -1331,10 +1317,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" t="s" s="2">
@@ -1351,26 +1337,24 @@
         <v>35</v>
       </c>
       <c r="I5" t="s" s="2">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="J5" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="L5" t="s" s="2">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="M5" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="N5" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="O5" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="O5" s="2"/>
       <c r="P5" t="s" s="2">
         <v>35</v>
       </c>
@@ -1382,7 +1366,7 @@
         <v>35</v>
       </c>
       <c r="T5" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="U5" t="s" s="2">
         <v>35</v>
@@ -1394,31 +1378,31 @@
         <v>35</v>
       </c>
       <c r="X5" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="Y5" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="Z5" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AA5" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AB5" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AC5" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AD5" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AE5" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AF5" t="s" s="2">
         <v>79</v>
-      </c>
-      <c r="Z5" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF5" t="s" s="2">
-        <v>70</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>36</v>
@@ -1433,24 +1417,24 @@
         <v>43</v>
       </c>
       <c r="AK5" t="s" s="2">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="AL5" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AM5" t="s" s="2">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="AN5" t="s" s="2">
-        <v>35</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1470,21 +1454,23 @@
         <v>35</v>
       </c>
       <c r="J6" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K6" t="s" s="2">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="L6" t="s" s="2">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="M6" t="s" s="2">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="N6" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="O6" s="2"/>
+        <v>91</v>
+      </c>
+      <c r="O6" t="s" s="2">
+        <v>92</v>
+      </c>
       <c r="P6" t="s" s="2">
         <v>35</v>
       </c>
@@ -1496,43 +1482,43 @@
         <v>35</v>
       </c>
       <c r="T6" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="U6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="V6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="W6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="X6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Y6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Z6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AA6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AB6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AC6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AD6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AE6" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AF6" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="U6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X6" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y6" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="Z6" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AA6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE6" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF6" t="s" s="2">
-        <v>84</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>36</v>
@@ -1547,24 +1533,24 @@
         <v>43</v>
       </c>
       <c r="AK6" t="s" s="2">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="AL6" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AM6" t="s" s="2">
         <v>35</v>
       </c>
       <c r="AN6" t="s" s="2">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1575,7 +1561,7 @@
         <v>36</v>
       </c>
       <c r="G7" t="s" s="2">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="H7" t="s" s="2">
         <v>35</v>
@@ -1584,23 +1570,21 @@
         <v>35</v>
       </c>
       <c r="J7" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K7" t="s" s="2">
         <v>48</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="N7" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="O7" t="s" s="2">
-        <v>97</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
         <v>35</v>
       </c>
@@ -1612,7 +1596,7 @@
         <v>35</v>
       </c>
       <c r="T7" t="s" s="2">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="U7" t="s" s="2">
         <v>35</v>
@@ -1648,13 +1632,13 @@
         <v>35</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH7" t="s" s="2">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="AI7" t="s" s="2">
         <v>42</v>
@@ -1663,35 +1647,35 @@
         <v>43</v>
       </c>
       <c r="AK7" t="s" s="2">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="AL7" t="s" s="2">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="AM7" t="s" s="2">
-        <v>35</v>
+        <v>104</v>
       </c>
       <c r="AN7" t="s" s="2">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
         <v>36</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H8" t="s" s="2">
         <v>35</v>
@@ -1700,19 +1684,19 @@
         <v>35</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K8" t="s" s="2">
         <v>48</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1726,49 +1710,49 @@
         <v>35</v>
       </c>
       <c r="T8" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="U8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="V8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="W8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="X8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Y8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Z8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AA8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AB8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AC8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AD8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AE8" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AF8" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="U8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF8" t="s" s="2">
-        <v>102</v>
-      </c>
       <c r="AG8" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>42</v>
@@ -1777,28 +1761,28 @@
         <v>43</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="AL8" t="s" s="2">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="AM8" t="s" s="2">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="AN8" t="s" s="2">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
@@ -1814,19 +1798,19 @@
         <v>35</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K9" t="s" s="2">
         <v>48</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="N9" t="s" s="2">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
@@ -1840,43 +1824,41 @@
         <v>35</v>
       </c>
       <c r="T9" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="U9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="V9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="W9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="X9" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="Y9" s="2"/>
+      <c r="Z9" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AA9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AB9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AC9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AD9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AE9" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AF9" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="U9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE9" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF9" t="s" s="2">
-        <v>111</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>36</v>
@@ -1891,28 +1873,28 @@
         <v>43</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="AL9" t="s" s="2">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="AM9" t="s" s="2">
-        <v>118</v>
+        <v>35</v>
       </c>
       <c r="AN9" t="s" s="2">
-        <v>119</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
@@ -1928,19 +1910,19 @@
         <v>35</v>
       </c>
       <c r="J10" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K10" t="s" s="2">
         <v>48</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="O10" s="2"/>
       <c r="P10" t="s" s="2">
@@ -1954,41 +1936,43 @@
         <v>35</v>
       </c>
       <c r="T10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="U10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="V10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="W10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="X10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Y10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Z10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AA10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AB10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AC10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AD10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AE10" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AF10" t="s" s="2">
         <v>125</v>
-      </c>
-      <c r="U10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X10" t="s" s="2">
-        <v>126</v>
-      </c>
-      <c r="Y10" s="2"/>
-      <c r="Z10" t="s" s="2">
-        <v>127</v>
-      </c>
-      <c r="AA10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE10" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF10" t="s" s="2">
-        <v>120</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>36</v>
@@ -2003,28 +1987,28 @@
         <v>43</v>
       </c>
       <c r="AK10" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AL10" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AM10" t="s" s="2">
-        <v>35</v>
+        <v>131</v>
       </c>
       <c r="AN10" t="s" s="2">
-        <v>35</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
@@ -2040,19 +2024,19 @@
         <v>35</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K11" t="s" s="2">
         <v>48</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="N11" t="s" s="2">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
@@ -2066,7 +2050,7 @@
         <v>35</v>
       </c>
       <c r="T11" t="s" s="2">
-        <v>35</v>
+        <v>137</v>
       </c>
       <c r="U11" t="s" s="2">
         <v>35</v>
@@ -2102,7 +2086,7 @@
         <v>35</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>36</v>
@@ -2117,28 +2101,28 @@
         <v>43</v>
       </c>
       <c r="AK11" t="s" s="2">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="AL11" t="s" s="2">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="AM11" t="s" s="2">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="AN11" t="s" s="2">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>139</v>
+        <v>35</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
@@ -2154,19 +2138,19 @@
         <v>35</v>
       </c>
       <c r="J12" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K12" t="s" s="2">
         <v>48</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="N12" t="s" s="2">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
@@ -2180,43 +2164,43 @@
         <v>35</v>
       </c>
       <c r="T12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="U12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="V12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="W12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="X12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Y12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="Z12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AA12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AB12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AC12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AD12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AE12" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="AF12" t="s" s="2">
         <v>142</v>
-      </c>
-      <c r="U12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE12" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF12" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>36</v>
@@ -2231,24 +2215,24 @@
         <v>43</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="AM12" t="s" s="2">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="AN12" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2268,21 +2252,23 @@
         <v>35</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>48</v>
+        <v>151</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="O13" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="O13" t="s" s="2">
+        <v>155</v>
+      </c>
       <c r="P13" t="s" s="2">
         <v>35</v>
       </c>
@@ -2294,7 +2280,7 @@
         <v>35</v>
       </c>
       <c r="T13" t="s" s="2">
-        <v>35</v>
+        <v>156</v>
       </c>
       <c r="U13" t="s" s="2">
         <v>35</v>
@@ -2330,7 +2316,7 @@
         <v>35</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>36</v>
@@ -2342,134 +2328,18 @@
         <v>42</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>43</v>
+        <v>157</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="AM13" t="s" s="2">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="B14" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G14" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="H14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J14" t="s" s="2">
-        <v>71</v>
-      </c>
-      <c r="K14" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="L14" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="N14" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="O14" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="P14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q14" s="2"/>
-      <c r="R14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T14" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="U14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE14" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF14" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="AG14" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH14" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="AI14" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AJ14" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AK14" t="s" s="2">
-        <v>163</v>
-      </c>
-      <c r="AL14" t="s" s="2">
-        <v>164</v>
-      </c>
-      <c r="AM14" t="s" s="2">
-        <v>165</v>
-      </c>
-      <c r="AN14" t="s" s="2">
         <v>35</v>
       </c>
     </row>

</xml_diff>